<commit_message>
Se añaden excepciones (obturadores)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://knorrbremsegroup-my.sharepoint.com/personal/david_gutierrez_merak-hvac_com/Documents/Dashboards/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="8_{8192E028-7CB0-4552-B695-D683C48028F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0672E47B-2741-4BF1-BC9C-8011256B01F5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FDB221-B9F2-4CD4-AFF1-C051B7F92399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>Botón personalizar columnas: cuando se pinche fuera de la ventana, ésta debe de cerrarse</t>
   </si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t>Sacar del código todas las rutas que apunten al Onedrive de KB porque cuando se haga la separación definitiva, se romperán los enlaces. Mejor opción en local: C:\users\"_&amp;_Environ$("USERNAME")_&amp;_"CARPETA". Modificar en VBA variable OutPath y htmlFull</t>
+  </si>
+  <si>
+    <t>Añadir imagen de herramientas necesarias con el resumen de los materiales en el modo gráfico / vision</t>
   </si>
 </sst>
 </file>
@@ -247,10 +250,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -571,7 +570,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF4DEE67-5682-410C-B7B8-D1B81A3E3B52}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="216.75" bestFit="1" customWidth="1"/>
@@ -765,6 +764,11 @@
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se sube fichero de prueba
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66FDB221-B9F2-4CD4-AFF1-C051B7F92399}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B28326B-35E7-4F16-97A6-D3D33A4E7D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
   <sheets>
     <sheet name="ICG VISION" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Botón personalizar columnas: cuando se pinche fuera de la ventana, ésta debe de cerrarse</t>
   </si>
@@ -185,6 +185,12 @@
   </si>
   <si>
     <t>Añadir imagen de herramientas necesarias con el resumen de los materiales en el modo gráfico / vision</t>
+  </si>
+  <si>
+    <t>Añadir la opción de abrir la imagen de los conectores terminados.</t>
+  </si>
+  <si>
+    <t>Que en el modo gráfico cuando se seleccione algún material de la lista, te resalte los cables en los que monta ese material</t>
   </si>
 </sst>
 </file>
@@ -199,7 +205,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -218,6 +224,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF33CC33"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -231,16 +243,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF33CC33"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -570,7 +588,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF4DEE67-5682-410C-B7B8-D1B81A3E3B52}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="216.75" bestFit="1" customWidth="1"/>
@@ -617,7 +635,7 @@
       </c>
     </row>
     <row r="9" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -732,7 +750,7 @@
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="A32" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -747,7 +765,7 @@
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="A35" s="3" t="s">
         <v>42</v>
       </c>
     </row>
@@ -769,6 +787,16 @@
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>47</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Versión 0.10.3 (Se corrige error en la interpretación de los decimales en el campo longitud)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B28326B-35E7-4F16-97A6-D3D33A4E7D65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F023CDC2-D944-4521-83C5-50CDBADFEF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
   <sheets>
     <sheet name="ICG VISION" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>Botón personalizar columnas: cuando se pinche fuera de la ventana, ésta debe de cerrarse</t>
   </si>
@@ -191,6 +191,12 @@
   </si>
   <si>
     <t>Que en el modo gráfico cuando se seleccione algún material de la lista, te resalte los cables en los que monta ese material</t>
+  </si>
+  <si>
+    <t>Añadir encabezado a los txt de los manguitos para que identifiquen la obra a la que pertenecen una vez impresos</t>
+  </si>
+  <si>
+    <t>Revisar el problema al crear el fichero txt para subir a sap que hace que la longitud de los cables no la tome bien cuando tiene decimales.</t>
   </si>
 </sst>
 </file>
@@ -205,7 +211,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -224,12 +230,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF33CC33"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -243,11 +243,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,7 +587,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF4DEE67-5682-410C-B7B8-D1B81A3E3B52}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="216.75" bestFit="1" customWidth="1"/>
@@ -750,7 +749,7 @@
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="1" t="s">
         <v>39</v>
       </c>
     </row>
@@ -765,7 +764,7 @@
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -797,6 +796,16 @@
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Versión 0.10.4 (Se corrige en el informe gráfico los cables que llegan del PC o de otro elemento y que no salen pintados porque no tienen código de cable)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F023CDC2-D944-4521-83C5-50CDBADFEF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF70C725-6F86-429F-B46E-4BE0CD2A03DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
+    <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
   <sheets>
     <sheet name="ICG VISION" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>Botón personalizar columnas: cuando se pinche fuera de la ventana, ésta debe de cerrarse</t>
   </si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t>Revisar el problema al crear el fichero txt para subir a sap que hace que la longitud de los cables no la tome bien cuando tiene decimales.</t>
+  </si>
+  <si>
+    <t>No se están pintando los cables que viene de Panel y van a un conector. Ver la lógica</t>
   </si>
 </sst>
 </file>
@@ -211,7 +214,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -230,6 +233,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF33CC33"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -243,10 +252,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -587,7 +597,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF4DEE67-5682-410C-B7B8-D1B81A3E3B52}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:A43"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="216.75" bestFit="1" customWidth="1"/>
@@ -653,159 +663,164 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+    <row r="15" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="16" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="19" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+    <row r="20" spans="1:1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
         <v>42</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="3" t="s">
         <v>51</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -815,6 +830,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E33343-36C6-4309-B345-C7F08FC9DB09}">
+  <sheetPr codeName="Hoja3"/>
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Versión 0.11.0 (Se añade que en la ventana de materiales del modo gráfico te permita iluminar el cable en el que monta cada material al seleccionarlo)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF70C725-6F86-429F-B46E-4BE0CD2A03DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C0575F-7E55-4191-9500-018CCB97DB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
@@ -199,7 +199,7 @@
     <t>Revisar el problema al crear el fichero txt para subir a sap que hace que la longitud de los cables no la tome bien cuando tiene decimales.</t>
   </si>
   <si>
-    <t>No se están pintando los cables que viene de Panel y van a un conector. Ver la lógica</t>
+    <t>No se están pintando los cables que viene de Panel y van a un conector. Ver la lógica. Corregido.</t>
   </si>
 </sst>
 </file>
@@ -819,7 +819,7 @@
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="3" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se sube archivo de mejoras
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77C0575F-7E55-4191-9500-018CCB97DB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898D27F6-4BF4-4B93-A095-2B4611167036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
@@ -214,7 +214,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,6 +239,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -252,11 +258,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,17 +796,17 @@
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="A38" s="4" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="A39" s="4" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="A40" s="4" t="s">
         <v>47</v>
       </c>
     </row>
@@ -809,7 +816,7 @@
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="A42" s="4" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Versión 0.13.1 (Se añaden terminales, herramientas)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{898D27F6-4BF4-4B93-A095-2B4611167036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA42DAC-4E98-4451-BEE3-2C638AFFAEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-15" windowWidth="29040" windowHeight="15720" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
   <sheets>
     <sheet name="ICG VISION" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>Botón personalizar columnas: cuando se pinche fuera de la ventana, ésta debe de cerrarse</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t>No se están pintando los cables que viene de Panel y van a un conector. Ver la lógica. Corregido.</t>
+  </si>
+  <si>
+    <t>No funciona el botón de copiar cuando filtras por ranking de proyectos.</t>
   </si>
 </sst>
 </file>
@@ -838,7 +841,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5E33343-36C6-4309-B345-C7F08FC9DB09}">
   <sheetPr codeName="Hoja3"/>
-  <dimension ref="A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="70.625" bestFit="1" customWidth="1"/>
@@ -847,6 +850,11 @@
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Versión 0.15.2 (corrección de errores de posicionamiento de iconos del la barra de herramientas)
</commit_message>
<xml_diff>
--- a/Mejoras.xlsx
+++ b/Mejoras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Produccion\DOI\PRODUCCION\Segmento PROTOTIPOS\IFA\David\Proyectos Visual Studio\ICG VISION\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFA42DAC-4E98-4451-BEE3-2C638AFFAEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DA61B9D-B23E-4B0C-8BC0-6307AFF3055A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{ABF5D909-D024-447E-B38E-40C6A21C1ED2}"/>
   </bookViews>
   <sheets>
     <sheet name="ICG VISION" sheetId="1" r:id="rId1"/>
@@ -853,7 +853,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>